<commit_message>
Atualização automática portal despesa
</commit_message>
<xml_diff>
--- a/upload/orgao2026.xlsx
+++ b/upload/orgao2026.xlsx
@@ -493,19 +493,19 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>22415131.08</v>
+        <v>22915657.51</v>
       </c>
       <c r="F2" t="n">
-        <v>16221742.57</v>
+        <v>16496274.91</v>
       </c>
       <c r="G2" t="n">
-        <v>14787594.36</v>
+        <v>14899520.38</v>
       </c>
       <c r="H2" t="n">
         <v>2727880.95</v>
       </c>
       <c r="I2" t="n">
-        <v>216944688.94</v>
+        <v>216945133.94</v>
       </c>
     </row>
     <row r="3">
@@ -526,13 +526,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1758306.07</v>
+        <v>1986291.21</v>
       </c>
       <c r="F3" t="n">
-        <v>1601588.54</v>
+        <v>1601658.7</v>
       </c>
       <c r="G3" t="n">
-        <v>1379722.12</v>
+        <v>1379790.37</v>
       </c>
       <c r="H3" t="n">
         <v>60903.67</v>
@@ -559,13 +559,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>178896103.47</v>
+        <v>178948067.63</v>
       </c>
       <c r="F4" t="n">
-        <v>109545332.47</v>
+        <v>110496155.24</v>
       </c>
       <c r="G4" t="n">
-        <v>98750058.11</v>
+        <v>99521480.12</v>
       </c>
       <c r="H4" t="n">
         <v>35391637.95</v>
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2860809.88</v>
+        <v>2861063.88</v>
       </c>
       <c r="F5" t="n">
-        <v>1710660.75</v>
+        <v>1762924.14</v>
       </c>
       <c r="G5" t="n">
-        <v>1473770.81</v>
+        <v>1523539.95</v>
       </c>
       <c r="H5" t="n">
         <v>706301.5699999999</v>
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2497227.64</v>
+        <v>2499067.64</v>
       </c>
       <c r="F6" t="n">
-        <v>1451380.33</v>
+        <v>1455598.88</v>
       </c>
       <c r="G6" t="n">
-        <v>1362028.33</v>
+        <v>1366243.16</v>
       </c>
       <c r="H6" t="n">
         <v>154717.57</v>
@@ -658,13 +658,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24811305.35</v>
+        <v>25002305.35</v>
       </c>
       <c r="F7" t="n">
-        <v>18556561.21</v>
+        <v>19790080.52</v>
       </c>
       <c r="G7" t="n">
-        <v>16731304.3</v>
+        <v>17519267.59</v>
       </c>
       <c r="H7" t="n">
         <v>2353030.07</v>
@@ -691,19 +691,19 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>77772291.09</v>
+        <v>79863957.14</v>
       </c>
       <c r="F8" t="n">
-        <v>30773321.07</v>
+        <v>33889776.63</v>
       </c>
       <c r="G8" t="n">
-        <v>27854296.19</v>
+        <v>29369112.68</v>
       </c>
       <c r="H8" t="n">
-        <v>45834152.39</v>
+        <v>51118822.19</v>
       </c>
       <c r="I8" t="n">
-        <v>47131914.41</v>
+        <v>49029933.96</v>
       </c>
     </row>
     <row r="9">
@@ -727,7 +727,7 @@
         <v>3484649.64</v>
       </c>
       <c r="F9" t="n">
-        <v>2695846.6</v>
+        <v>2700019.98</v>
       </c>
       <c r="G9" t="n">
         <v>2602959.85</v>
@@ -757,19 +757,19 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>81849575.48999999</v>
+        <v>83451344.81</v>
       </c>
       <c r="F10" t="n">
-        <v>72661047.7</v>
+        <v>76749035.73999999</v>
       </c>
       <c r="G10" t="n">
-        <v>63546344.13</v>
+        <v>64331542.04</v>
       </c>
       <c r="H10" t="n">
         <v>14925708.98</v>
       </c>
       <c r="I10" t="n">
-        <v>13881706.51</v>
+        <v>13889226.51</v>
       </c>
     </row>
     <row r="11">
@@ -790,19 +790,19 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1561236884.63</v>
+        <v>1621116303.32</v>
       </c>
       <c r="F11" t="n">
-        <v>824490142.15</v>
+        <v>834816709.8</v>
       </c>
       <c r="G11" t="n">
-        <v>797316689.8200001</v>
+        <v>814730941.02</v>
       </c>
       <c r="H11" t="n">
-        <v>334598887.77</v>
+        <v>338223224.55</v>
       </c>
       <c r="I11" t="n">
-        <v>340409119.02</v>
+        <v>342813777.57</v>
       </c>
     </row>
     <row r="12">
@@ -823,13 +823,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>33881959.45</v>
+        <v>34227344.15</v>
       </c>
       <c r="F12" t="n">
-        <v>10198029.11</v>
+        <v>10340289.26</v>
       </c>
       <c r="G12" t="n">
-        <v>9409144.609999999</v>
+        <v>9542932.08</v>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
@@ -918,13 +918,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>210407094.06</v>
+        <v>243357094.6</v>
       </c>
       <c r="F15" t="n">
-        <v>210407094.06</v>
+        <v>243357094.6</v>
       </c>
       <c r="G15" t="n">
-        <v>210407094.06</v>
+        <v>243357094.6</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>17658291.2</v>
+        <v>19634354.31</v>
       </c>
       <c r="F16" t="n">
-        <v>17658291.2</v>
+        <v>19634354.31</v>
       </c>
       <c r="G16" t="n">
-        <v>17658291.2</v>
+        <v>19634354.31</v>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -999,13 +999,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>85431443.5</v>
+        <v>98640447.63</v>
       </c>
       <c r="F18" t="n">
-        <v>85431443.5</v>
+        <v>98640447.63</v>
       </c>
       <c r="G18" t="n">
-        <v>85431443.5</v>
+        <v>98640447.63</v>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -1028,13 +1028,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>8645474.49</v>
+        <v>8668649.49</v>
       </c>
       <c r="F19" t="n">
-        <v>4390380.98</v>
+        <v>4402544.98</v>
       </c>
       <c r="G19" t="n">
-        <v>4020702.75</v>
+        <v>4030056.44</v>
       </c>
       <c r="H19" t="n">
         <v>1040158.72</v>
@@ -1064,10 +1064,10 @@
         <v>358206</v>
       </c>
       <c r="F20" t="n">
-        <v>212512.09</v>
+        <v>223427.58</v>
       </c>
       <c r="G20" t="n">
-        <v>200780.62</v>
+        <v>211696.11</v>
       </c>
       <c r="H20" t="n">
         <v>30324.78</v>
@@ -1094,13 +1094,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>918523.89</v>
+        <v>1004317.92</v>
       </c>
       <c r="F21" t="n">
-        <v>749432.03</v>
+        <v>838104.04</v>
       </c>
       <c r="G21" t="n">
-        <v>621295.3</v>
+        <v>693062.3</v>
       </c>
       <c r="H21" t="n">
         <v>97349.38</v>
@@ -1127,13 +1127,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>19082553.74</v>
+        <v>19017448.76</v>
       </c>
       <c r="F22" t="n">
-        <v>16420623.95</v>
+        <v>16485291.12</v>
       </c>
       <c r="G22" t="n">
-        <v>14435895.25</v>
+        <v>14689413.44</v>
       </c>
       <c r="H22" t="n">
         <v>4345882.84</v>
@@ -1160,13 +1160,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>8853290.779999999</v>
+        <v>8970870.439999999</v>
       </c>
       <c r="F23" t="n">
-        <v>7943980.07</v>
+        <v>8009583.65</v>
       </c>
       <c r="G23" t="n">
-        <v>6994334.95</v>
+        <v>7062983.28</v>
       </c>
       <c r="H23" t="n">
         <v>1741057.76</v>
@@ -1202,10 +1202,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1921024.46</v>
+        <v>2122233.46</v>
       </c>
       <c r="I24" t="n">
-        <v>1828815.27</v>
+        <v>2020366.24</v>
       </c>
     </row>
     <row r="25">
@@ -1255,13 +1255,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>11010371.13</v>
+        <v>11280695.13</v>
       </c>
       <c r="F26" t="n">
-        <v>4402545.3</v>
+        <v>4407081.74</v>
       </c>
       <c r="G26" t="n">
-        <v>4352573.91</v>
+        <v>4357523.1</v>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>9417855.18</v>
+        <v>9829781.16</v>
       </c>
       <c r="F27" t="n">
-        <v>9060070.529999999</v>
+        <v>9424323.33</v>
       </c>
       <c r="G27" t="n">
-        <v>7626121.2</v>
+        <v>7650353.71</v>
       </c>
       <c r="H27" t="n">
         <v>1102595.36</v>
@@ -1317,13 +1317,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>8382802.49</v>
+        <v>9063969.41</v>
       </c>
       <c r="F28" t="n">
-        <v>7013936.1</v>
+        <v>7103215.07</v>
       </c>
       <c r="G28" t="n">
-        <v>6297041.02</v>
+        <v>6301286.12</v>
       </c>
       <c r="H28" t="n">
         <v>1499694.06</v>
@@ -1377,13 +1377,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2719324.85</v>
+        <v>3020706.72</v>
       </c>
       <c r="F30" t="n">
-        <v>1943303.29</v>
+        <v>1946792.06</v>
       </c>
       <c r="G30" t="n">
-        <v>1346017.29</v>
+        <v>1891769.63</v>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
@@ -1460,10 +1460,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>14088679.2</v>
+        <v>14089679.2</v>
       </c>
       <c r="F33" t="n">
-        <v>10150334.06</v>
+        <v>10218932.06</v>
       </c>
       <c r="G33" t="n">
         <v>9109782.140000001</v>
@@ -1493,19 +1493,19 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1435771676.37</v>
+        <v>1451036701.01</v>
       </c>
       <c r="F34" t="n">
-        <v>1092570706.34</v>
+        <v>1097251187.75</v>
       </c>
       <c r="G34" t="n">
-        <v>940775249.28</v>
+        <v>945472044.86</v>
       </c>
       <c r="H34" t="n">
-        <v>264060155.38</v>
+        <v>268651744.87</v>
       </c>
       <c r="I34" t="n">
-        <v>245461898.29</v>
+        <v>249998388.71</v>
       </c>
     </row>
     <row r="35">
@@ -1526,19 +1526,19 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>929143919.91</v>
+        <v>948700388.71</v>
       </c>
       <c r="F35" t="n">
-        <v>564219521.16</v>
+        <v>573559413.83</v>
       </c>
       <c r="G35" t="n">
-        <v>486997835.23</v>
+        <v>504906661.32</v>
       </c>
       <c r="H35" t="n">
-        <v>567287208.3099999</v>
+        <v>571796224.36</v>
       </c>
       <c r="I35" t="n">
-        <v>1012471891.58</v>
+        <v>1021423931.1</v>
       </c>
     </row>
     <row r="36">
@@ -1559,19 +1559,19 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>42544902.07</v>
+        <v>43964830.52</v>
       </c>
       <c r="F36" t="n">
-        <v>12997497.91</v>
+        <v>13469389.17</v>
       </c>
       <c r="G36" t="n">
-        <v>10966232.21</v>
+        <v>11318552.03</v>
       </c>
       <c r="H36" t="n">
-        <v>38712818.59</v>
+        <v>39907351.55</v>
       </c>
       <c r="I36" t="n">
-        <v>43751685.05</v>
+        <v>45095365.05</v>
       </c>
     </row>
     <row r="37">
@@ -1592,13 +1592,13 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>389537.41</v>
+        <v>411364.79</v>
       </c>
       <c r="F37" t="n">
-        <v>325505.69</v>
+        <v>325783.39</v>
       </c>
       <c r="G37" t="n">
-        <v>304680.58</v>
+        <v>304944.95</v>
       </c>
       <c r="H37" t="n">
         <v>1251438.8</v>
@@ -1652,13 +1652,13 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>16375111.89</v>
+        <v>16440845.32</v>
       </c>
       <c r="F39" t="n">
-        <v>10834096.17</v>
+        <v>10948901.45</v>
       </c>
       <c r="G39" t="n">
-        <v>10372955.07</v>
+        <v>10481085.4</v>
       </c>
       <c r="H39" t="n">
         <v>2161550.53</v>
@@ -1685,19 +1685,19 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>478341486.01</v>
+        <v>487480867.19</v>
       </c>
       <c r="F40" t="n">
-        <v>381087576.67</v>
+        <v>400121836.41</v>
       </c>
       <c r="G40" t="n">
-        <v>342890753.62</v>
+        <v>347218239.44</v>
       </c>
       <c r="H40" t="n">
-        <v>99508258.3</v>
+        <v>99726449.48999999</v>
       </c>
       <c r="I40" t="n">
-        <v>100084193.41</v>
+        <v>100468044.69</v>
       </c>
     </row>
     <row r="41">
@@ -1721,10 +1721,10 @@
         <v>222775.76</v>
       </c>
       <c r="F41" t="n">
-        <v>195711.57</v>
+        <v>222775.76</v>
       </c>
       <c r="G41" t="n">
-        <v>164479.93</v>
+        <v>186763.97</v>
       </c>
       <c r="H41" t="n">
         <v>842769.0699999999</v>
@@ -1781,10 +1781,10 @@
         <v>8163868.5</v>
       </c>
       <c r="F43" t="n">
-        <v>6300081.39</v>
+        <v>6305142.86</v>
       </c>
       <c r="G43" t="n">
-        <v>5457103.79</v>
+        <v>5537225.6</v>
       </c>
       <c r="H43" t="n">
         <v>2576363.8</v>
@@ -1877,13 +1877,13 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1480644.25</v>
+        <v>1497423.85</v>
       </c>
       <c r="F46" t="n">
-        <v>967430.05</v>
+        <v>1039016.09</v>
       </c>
       <c r="G46" t="n">
-        <v>874286.28</v>
+        <v>928627.59</v>
       </c>
       <c r="H46" t="n">
         <v>178281.27</v>
@@ -1964,16 +1964,16 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>211040578.99</v>
+        <v>213940137.6</v>
       </c>
       <c r="F49" t="n">
-        <v>146406584.76</v>
+        <v>150326749.26</v>
       </c>
       <c r="G49" t="n">
-        <v>129579455.13</v>
+        <v>130396590.8</v>
       </c>
       <c r="H49" t="n">
-        <v>135331229.29</v>
+        <v>135331656.77</v>
       </c>
       <c r="I49" t="n">
         <v>141000459.38</v>
@@ -2006,10 +2006,10 @@
         <v>14173841.97</v>
       </c>
       <c r="H50" t="n">
-        <v>19810018.83</v>
+        <v>19810614.22</v>
       </c>
       <c r="I50" t="n">
-        <v>21159454.29</v>
+        <v>21159895.87</v>
       </c>
     </row>
     <row r="51">
@@ -2030,13 +2030,13 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>94044732.23</v>
+        <v>97629701.23</v>
       </c>
       <c r="F51" t="n">
-        <v>57882497.43</v>
+        <v>59057477.35</v>
       </c>
       <c r="G51" t="n">
-        <v>54816106.12</v>
+        <v>54987294.69</v>
       </c>
       <c r="H51" t="n">
         <v>18617499.53</v>
@@ -2063,13 +2063,13 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>48405402.56</v>
+        <v>49429749.1</v>
       </c>
       <c r="F52" t="n">
-        <v>21206390.26</v>
+        <v>21468657.17</v>
       </c>
       <c r="G52" t="n">
-        <v>18506076.14</v>
+        <v>18964753.93</v>
       </c>
       <c r="H52" t="n">
         <v>12470050.72</v>
@@ -2123,13 +2123,13 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>142871780.64</v>
+        <v>146396072.66</v>
       </c>
       <c r="F54" t="n">
-        <v>109643004.49</v>
+        <v>111890906.46</v>
       </c>
       <c r="G54" t="n">
-        <v>98165742.48</v>
+        <v>98317974.44</v>
       </c>
       <c r="H54" t="n">
         <v>24490691.01</v>
@@ -2156,19 +2156,19 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>29409821.91</v>
+        <v>29810353.41</v>
       </c>
       <c r="F55" t="n">
-        <v>21545152.47</v>
+        <v>21643916.29</v>
       </c>
       <c r="G55" t="n">
-        <v>20722017.78</v>
+        <v>20985661.34</v>
       </c>
       <c r="H55" t="n">
-        <v>22118707.18</v>
+        <v>22140382.18</v>
       </c>
       <c r="I55" t="n">
-        <v>22868744.96</v>
+        <v>22890160.12</v>
       </c>
     </row>
     <row r="56">
@@ -2189,13 +2189,13 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>44031959.61</v>
+        <v>45995878.1</v>
       </c>
       <c r="F56" t="n">
-        <v>36904199.49</v>
+        <v>39054421.46</v>
       </c>
       <c r="G56" t="n">
-        <v>31023491.7</v>
+        <v>31924889.43</v>
       </c>
       <c r="H56" t="n">
         <v>8627975.140000001</v>
@@ -2222,13 +2222,13 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>4266882.26</v>
+        <v>4667411.74</v>
       </c>
       <c r="F57" t="n">
-        <v>3546927.07</v>
+        <v>3960220.12</v>
       </c>
       <c r="G57" t="n">
-        <v>3173108.8</v>
+        <v>3228548.32</v>
       </c>
       <c r="H57" t="n">
         <v>532120.09</v>
@@ -2255,13 +2255,13 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>6719534.81</v>
+        <v>6995627.38</v>
       </c>
       <c r="F58" t="n">
-        <v>4597087.66</v>
+        <v>4879204.46</v>
       </c>
       <c r="G58" t="n">
-        <v>4320007.08</v>
+        <v>4559527.17</v>
       </c>
       <c r="H58" t="n">
         <v>11029049.85</v>
@@ -2288,13 +2288,13 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>14861291.68</v>
+        <v>14985968.97</v>
       </c>
       <c r="F59" t="n">
-        <v>8433425.58</v>
+        <v>8751519.33</v>
       </c>
       <c r="G59" t="n">
-        <v>7571977.46</v>
+        <v>7610772.22</v>
       </c>
       <c r="H59" t="n">
         <v>5237570.34</v>
@@ -2321,13 +2321,13 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>9262595.25</v>
+        <v>9543644.470000001</v>
       </c>
       <c r="F60" t="n">
-        <v>9017803.58</v>
+        <v>9291129.300000001</v>
       </c>
       <c r="G60" t="n">
-        <v>7916640.25</v>
+        <v>8173772.91</v>
       </c>
       <c r="H60" t="n">
         <v>1332496.42</v>
@@ -2354,13 +2354,13 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>42043986.36</v>
+        <v>47222671.95</v>
       </c>
       <c r="F61" t="n">
-        <v>42043986.36</v>
+        <v>47222671.95</v>
       </c>
       <c r="G61" t="n">
-        <v>42043986.36</v>
+        <v>47222671.95</v>
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
@@ -2383,19 +2383,19 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>236204307.71</v>
+        <v>238917109.87</v>
       </c>
       <c r="F62" t="n">
-        <v>184849969.63</v>
+        <v>193375069.51</v>
       </c>
       <c r="G62" t="n">
-        <v>170020318.08</v>
+        <v>179475084.47</v>
       </c>
       <c r="H62" t="n">
-        <v>198983832.99</v>
+        <v>199055061.08</v>
       </c>
       <c r="I62" t="n">
-        <v>194272748.12</v>
+        <v>194341491.84</v>
       </c>
     </row>
     <row r="63">
@@ -2416,19 +2416,19 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>67828383.36</v>
+        <v>66845383.36</v>
       </c>
       <c r="F63" t="n">
-        <v>48384727.31</v>
+        <v>53539938.46</v>
       </c>
       <c r="G63" t="n">
-        <v>43905078.36</v>
+        <v>43974097.76</v>
       </c>
       <c r="H63" t="n">
-        <v>35392114.99</v>
+        <v>35392441.77</v>
       </c>
       <c r="I63" t="n">
-        <v>53898519.67</v>
+        <v>53934542.42</v>
       </c>
     </row>
     <row r="64">
@@ -2449,13 +2449,13 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>11541979.66</v>
+        <v>11607890.08</v>
       </c>
       <c r="F64" t="n">
         <v>8064558.63</v>
       </c>
       <c r="G64" t="n">
-        <v>6925082.61</v>
+        <v>7591360.75</v>
       </c>
       <c r="H64" t="n">
         <v>1960878.57</v>
@@ -2485,10 +2485,10 @@
         <v>584746.91</v>
       </c>
       <c r="F65" t="n">
-        <v>468155.48</v>
+        <v>561739.67</v>
       </c>
       <c r="G65" t="n">
-        <v>405609.52</v>
+        <v>484972.44</v>
       </c>
       <c r="H65" t="n">
         <v>34744.58</v>
@@ -2542,7 +2542,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1470240.61</v>
+        <v>1474364.46</v>
       </c>
       <c r="F67" t="n">
         <v>1193299.64</v>
@@ -2551,10 +2551,10 @@
         <v>1103997.51</v>
       </c>
       <c r="H67" t="n">
-        <v>94459.97</v>
+        <v>94595.71000000001</v>
       </c>
       <c r="I67" t="n">
-        <v>93457.72</v>
+        <v>93586.94</v>
       </c>
     </row>
     <row r="68">
@@ -2575,19 +2575,19 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>234786515.26</v>
+        <v>246468987.84</v>
       </c>
       <c r="F68" t="n">
-        <v>171889919.57</v>
+        <v>187529645.68</v>
       </c>
       <c r="G68" t="n">
-        <v>151772993.4</v>
+        <v>153213333.12</v>
       </c>
       <c r="H68" t="n">
-        <v>49463492.27</v>
+        <v>49474619.75</v>
       </c>
       <c r="I68" t="n">
-        <v>48253127.95</v>
+        <v>48319062.06</v>
       </c>
     </row>
     <row r="69">
@@ -2608,19 +2608,19 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>260710928.02</v>
+        <v>270265210.42</v>
       </c>
       <c r="F69" t="n">
-        <v>194028271.69</v>
+        <v>196511634.68</v>
       </c>
       <c r="G69" t="n">
-        <v>166810496.62</v>
+        <v>168933198.89</v>
       </c>
       <c r="H69" t="n">
-        <v>88100410.09</v>
+        <v>88100522.73999999</v>
       </c>
       <c r="I69" t="n">
-        <v>84956671.15000001</v>
+        <v>84956779.47</v>
       </c>
     </row>
     <row r="70">
@@ -2641,19 +2641,19 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>485810309.21</v>
+        <v>494652449.31</v>
       </c>
       <c r="F70" t="n">
-        <v>303996284.61</v>
+        <v>312050998.41</v>
       </c>
       <c r="G70" t="n">
-        <v>267816295.82</v>
+        <v>277120152.85</v>
       </c>
       <c r="H70" t="n">
-        <v>235557840.68</v>
+        <v>235618798.54</v>
       </c>
       <c r="I70" t="n">
-        <v>205152026.49</v>
+        <v>205259183.86</v>
       </c>
     </row>
     <row r="71">
@@ -2677,10 +2677,10 @@
         <v>1086537.57</v>
       </c>
       <c r="F71" t="n">
-        <v>986783.6800000001</v>
+        <v>1063747.56</v>
       </c>
       <c r="G71" t="n">
-        <v>880176.9300000001</v>
+        <v>924442.6899999999</v>
       </c>
       <c r="H71" t="n">
         <v>225243.01</v>
@@ -2707,13 +2707,13 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>58978647.59</v>
+        <v>59110548.59</v>
       </c>
       <c r="F72" t="n">
-        <v>38585801.96</v>
+        <v>38630645.31</v>
       </c>
       <c r="G72" t="n">
-        <v>37118035.4</v>
+        <v>37160449.89</v>
       </c>
       <c r="H72" t="n">
         <v>19489131.64</v>
@@ -2740,13 +2740,13 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>1732099.9</v>
+        <v>1784536.37</v>
       </c>
       <c r="F73" t="n">
-        <v>1398181.53</v>
+        <v>1557406.41</v>
       </c>
       <c r="G73" t="n">
-        <v>1233215.85</v>
+        <v>1335480.21</v>
       </c>
       <c r="H73" t="n">
         <v>34378.25</v>
@@ -2773,19 +2773,19 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>79403938.59</v>
+        <v>91161042.12</v>
       </c>
       <c r="F74" t="n">
-        <v>64175278.12</v>
+        <v>65227308.63</v>
       </c>
       <c r="G74" t="n">
-        <v>60217584.82</v>
+        <v>61234742.26</v>
       </c>
       <c r="H74" t="n">
-        <v>66007855.09</v>
+        <v>66745461.28</v>
       </c>
       <c r="I74" t="n">
-        <v>62689623.1</v>
+        <v>62742403.58</v>
       </c>
     </row>
     <row r="75">
@@ -2806,13 +2806,13 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>19256664.18</v>
+        <v>19270546.18</v>
       </c>
       <c r="F75" t="n">
-        <v>15178006.27</v>
+        <v>16266161</v>
       </c>
       <c r="G75" t="n">
-        <v>12006129.05</v>
+        <v>13485858.86</v>
       </c>
       <c r="H75" t="n">
         <v>674995.91</v>
@@ -2839,16 +2839,16 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>242899915.51</v>
+        <v>242952007.51</v>
       </c>
       <c r="F76" t="n">
-        <v>11725453.81</v>
+        <v>13179804.85</v>
       </c>
       <c r="G76" t="n">
-        <v>10427477.65</v>
+        <v>11510927.08</v>
       </c>
       <c r="H76" t="n">
-        <v>50036034.12</v>
+        <v>50585699.32</v>
       </c>
       <c r="I76" t="n">
         <v>47319399.62</v>
@@ -2872,19 +2872,19 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>26313213.94</v>
+        <v>26607344.26</v>
       </c>
       <c r="F77" t="n">
-        <v>21575294.77</v>
+        <v>22085520.18</v>
       </c>
       <c r="G77" t="n">
-        <v>17870272.12</v>
+        <v>19744337.53</v>
       </c>
       <c r="H77" t="n">
-        <v>18126905.4</v>
+        <v>18154376.27</v>
       </c>
       <c r="I77" t="n">
-        <v>29279133.49</v>
+        <v>29303994.63</v>
       </c>
     </row>
     <row r="78">
@@ -2905,19 +2905,19 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>953992229.74</v>
+        <v>970087628.3099999</v>
       </c>
       <c r="F78" t="n">
-        <v>723891311.2</v>
+        <v>739096255.62</v>
       </c>
       <c r="G78" t="n">
-        <v>698450457.41</v>
+        <v>713367442.08</v>
       </c>
       <c r="H78" t="n">
-        <v>155884404.2</v>
+        <v>157440192.63</v>
       </c>
       <c r="I78" t="n">
-        <v>351009889.12</v>
+        <v>352178826.45</v>
       </c>
     </row>
     <row r="79">
@@ -2938,19 +2938,19 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>182912408.42</v>
+        <v>189602554.73</v>
       </c>
       <c r="F79" t="n">
-        <v>134834701.28</v>
+        <v>138321317.18</v>
       </c>
       <c r="G79" t="n">
-        <v>107583959.85</v>
+        <v>107916254.16</v>
       </c>
       <c r="H79" t="n">
         <v>62673101.03</v>
       </c>
       <c r="I79" t="n">
-        <v>66670976.86</v>
+        <v>66788140.89</v>
       </c>
     </row>
     <row r="80">
@@ -2971,13 +2971,13 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>30538470.74</v>
+        <v>30864031.14</v>
       </c>
       <c r="F80" t="n">
-        <v>26673915.73</v>
+        <v>27066019.4</v>
       </c>
       <c r="G80" t="n">
-        <v>24684840.67</v>
+        <v>24770980.49</v>
       </c>
       <c r="H80" t="n">
         <v>4983225.57</v>
@@ -3004,16 +3004,16 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>53609808.85</v>
+        <v>53720447.55</v>
       </c>
       <c r="F81" t="n">
-        <v>29669424.88</v>
+        <v>30520466.38</v>
       </c>
       <c r="G81" t="n">
-        <v>26613915.68</v>
+        <v>26978325.24</v>
       </c>
       <c r="H81" t="n">
-        <v>92783753.01000001</v>
+        <v>93035965.29000001</v>
       </c>
       <c r="I81" t="n">
         <v>149841879.2</v>
@@ -3037,19 +3037,19 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>606278842.4400001</v>
+        <v>610001632.2</v>
       </c>
       <c r="F82" t="n">
-        <v>446204838.77</v>
+        <v>451888200.92</v>
       </c>
       <c r="G82" t="n">
-        <v>422722271.24</v>
+        <v>428692401.42</v>
       </c>
       <c r="H82" t="n">
-        <v>144895064.91</v>
+        <v>145105621.93</v>
       </c>
       <c r="I82" t="n">
-        <v>152004702.77</v>
+        <v>152617812.4</v>
       </c>
     </row>
     <row r="83">
@@ -3070,13 +3070,13 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>31512844.84</v>
+        <v>31743384.51</v>
       </c>
       <c r="F83" t="n">
-        <v>26993582.24</v>
+        <v>27291253.35</v>
       </c>
       <c r="G83" t="n">
-        <v>20987360.64</v>
+        <v>23579319.56</v>
       </c>
       <c r="H83" t="n">
         <v>4788552.39</v>
@@ -3103,19 +3103,19 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>284016956.71</v>
+        <v>283562979.71</v>
       </c>
       <c r="F84" t="n">
-        <v>207719080.21</v>
+        <v>216285129.65</v>
       </c>
       <c r="G84" t="n">
-        <v>186399379.79</v>
+        <v>188584148.63</v>
       </c>
       <c r="H84" t="n">
         <v>74964907.94</v>
       </c>
       <c r="I84" t="n">
-        <v>100438151.39</v>
+        <v>99677843.55</v>
       </c>
     </row>
     <row r="85">
@@ -3136,19 +3136,19 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>94483925.47</v>
+        <v>95543759.13</v>
       </c>
       <c r="F85" t="n">
-        <v>69372102.87</v>
+        <v>70049664.89</v>
       </c>
       <c r="G85" t="n">
-        <v>58646143.53</v>
+        <v>59149824.92</v>
       </c>
       <c r="H85" t="n">
-        <v>34226175.48</v>
+        <v>34371578.38</v>
       </c>
       <c r="I85" t="n">
-        <v>29952557.14</v>
+        <v>30087345.63</v>
       </c>
     </row>
     <row r="86">
@@ -3169,13 +3169,13 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>9992152.27</v>
+        <v>10099744.05</v>
       </c>
       <c r="F86" t="n">
-        <v>8249961.66</v>
+        <v>8427815.470000001</v>
       </c>
       <c r="G86" t="n">
-        <v>7420904.84</v>
+        <v>7504646.16</v>
       </c>
       <c r="H86" t="n">
         <v>5342633.4</v>
@@ -3202,10 +3202,10 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>5543851.35</v>
+        <v>5662062.43</v>
       </c>
       <c r="F87" t="n">
-        <v>4292556.54</v>
+        <v>4760884.23</v>
       </c>
       <c r="G87" t="n">
         <v>3036744.6</v>
@@ -3235,19 +3235,19 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>66762770.06</v>
+        <v>68528819.48999999</v>
       </c>
       <c r="F88" t="n">
-        <v>48062788.92</v>
+        <v>48467299.88</v>
       </c>
       <c r="G88" t="n">
-        <v>42846124.83</v>
+        <v>43141302.15</v>
       </c>
       <c r="H88" t="n">
-        <v>20790290.67</v>
+        <v>20790468.79</v>
       </c>
       <c r="I88" t="n">
-        <v>19991976.69</v>
+        <v>19992125.98</v>
       </c>
     </row>
     <row r="89">
@@ -3268,19 +3268,19 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>57160466.52</v>
+        <v>57419511.15</v>
       </c>
       <c r="F89" t="n">
-        <v>38069320.72</v>
+        <v>41113437.23</v>
       </c>
       <c r="G89" t="n">
-        <v>34126736.11</v>
+        <v>36756683.13</v>
       </c>
       <c r="H89" t="n">
-        <v>25670879.72</v>
+        <v>25671551.83</v>
       </c>
       <c r="I89" t="n">
-        <v>23665823.26</v>
+        <v>23666371.42</v>
       </c>
     </row>
     <row r="90">
@@ -3301,13 +3301,13 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>2321177.78</v>
+        <v>2351482.68</v>
       </c>
       <c r="F90" t="n">
-        <v>2069207.73</v>
+        <v>2086137.58</v>
       </c>
       <c r="G90" t="n">
-        <v>1815836.86</v>
+        <v>1832442.34</v>
       </c>
       <c r="H90" t="n">
         <v>294468.9</v>

</xml_diff>